<commit_message>
update to run on VM
</commit_message>
<xml_diff>
--- a/_Voorbereiding_Python/_waterkwantiteit/define_parameter_selection.xlsx
+++ b/_Voorbereiding_Python/_waterkwantiteit/define_parameter_selection.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projecten\RWS\DigSysRapWadden\_Voorbereiding_Python\_waterkwantiteit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CE3234E-070E-4D94-BD18-7E9DF8662ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4835A713-F62B-49BC-9035-3B52ABD8F11B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="135" yWindow="3030" windowWidth="21600" windowHeight="12525" xr2:uid="{92CF524D-9381-4F13-A4CC-44084FD21FA3}"/>
+    <workbookView xWindow="2530" yWindow="1370" windowWidth="14400" windowHeight="8170" xr2:uid="{92CF524D-9381-4F13-A4CC-44084FD21FA3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="7">
   <si>
     <t>ProcesType</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>NAP</t>
+  </si>
+  <si>
+    <t>astronomisch</t>
   </si>
 </sst>
 </file>
@@ -428,10 +431,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8793A05-AA6D-4227-ACD5-5212AE36C656}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -442,7 +445,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -450,6 +453,17 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>